<commit_message>
Updated KEN_grids_kan10 model - 2026-06-18 23:38
</commit_message>
<xml_diff>
--- a/VerveStacks_KEN_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_KEN_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_KEN_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{06A451C2-9C8B-435A-B818-368711C0B667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CD080AE-F5D3-4150-961C-CEF602F02F53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22656,7 +22656,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48AA1C7F-1178-4DCE-B438-5E0A01DE28EC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84D8764B-1CF8-4AFC-82F4-58F09CF16B3A}">
   <dimension ref="B9:H83"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -24154,7 +24154,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9A9215-0C36-499C-9834-1E82D8FD0464}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46CE7619-038C-4CD9-A133-D25107D1E584}">
   <dimension ref="B9:L83"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>